<commit_message>
Refactor Hino 2-lane tests and introduce wraparound scheduling logic
- Updated test suite for Hino 2-lane scheduling to reflect new wraparound behavior.
- Added new tests for Hino 2-lane wraparound scenarios, ensuring correct start times based on previous bins.
- Removed legacy tests and refactored existing ones to align with new implementation.
- Introduced helper functions for processing details and master data.
- Ensured backward compatibility for non-Hino vendors and existing logic.
- Updated constants and imports in the sorter tests to accommodate new functionality.
- Modified Excel file related to Hino scheduling to reflect changes.
</commit_message>
<xml_diff>
--- a/入車時間マスタ.xlsx
+++ b/入車時間マスタ.xlsx
@@ -466,11 +466,7 @@
           <t>06:25</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -488,11 +484,7 @@
           <t>14:31</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -510,11 +502,7 @@
           <t>08:16</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -532,11 +520,7 @@
           <t>10:56</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -554,11 +538,7 @@
           <t>14:11</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -576,11 +556,7 @@
           <t>17:53</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -598,11 +574,7 @@
           <t>21:34</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -620,11 +592,7 @@
           <t>00:09</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -642,11 +610,7 @@
           <t>19:55</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -664,11 +628,7 @@
           <t>07:10</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="D11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -686,11 +646,7 @@
           <t>11:25</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -708,11 +664,7 @@
           <t>17:30</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -730,11 +682,7 @@
           <t>22:00</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -749,14 +697,10 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>07:34</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+          <t>23:19</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -771,14 +715,10 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>13:01</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+          <t>07:34</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -793,14 +733,10 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>17:16</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>13:01</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -815,14 +751,10 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>23:19</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+          <t>17:16</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -837,14 +769,10 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>06:29</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>16:59</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -859,14 +787,10 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>07:54</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -881,14 +805,10 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>09:02</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+          <t>19:39</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -903,14 +823,10 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>09:54</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+          <t>21:18</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -925,14 +841,10 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>12:00</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+          <t>22:20</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -947,14 +859,10 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>12:45</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+          <t>23:50</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -969,14 +877,10 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>13:52</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+          <t>00:24</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -991,14 +895,10 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>14:59</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+          <t>06:29</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1013,14 +913,10 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>16:59</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>07:54</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1035,14 +931,10 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>18:30</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+          <t>09:02</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1057,14 +949,10 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>19:39</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+          <t>09:54</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1079,14 +967,10 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>21:18</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1101,14 +985,10 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>22:20</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+          <t>12:45</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1123,14 +1003,10 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>23:50</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+          <t>13:52</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1145,14 +1021,10 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>00:24</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+          <t>14:59</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1170,11 +1042,7 @@
           <t>10:10</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1184,7 +1052,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>03</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1192,11 +1060,7 @@
           <t>08:30</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1206,7 +1070,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>02</t>
+          <t>04</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1214,11 +1078,7 @@
           <t>10:30</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1228,7 +1088,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>03</t>
+          <t>05</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1236,11 +1096,7 @@
           <t>12:30</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1250,7 +1106,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>04</t>
+          <t>06</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1258,11 +1114,7 @@
           <t>16:00</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1272,7 +1124,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>05</t>
+          <t>07</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1280,11 +1132,7 @@
           <t>18:15</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1294,7 +1142,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>06</t>
+          <t>08</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1302,11 +1150,7 @@
           <t>20:35</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1316,7 +1160,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>07</t>
+          <t>01</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1324,11 +1168,7 @@
           <t>23:35</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1338,7 +1178,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>08</t>
+          <t>02</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1346,11 +1186,7 @@
           <t>01:00</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1368,11 +1204,7 @@
           <t>11:40</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1390,11 +1222,7 @@
           <t>00:40</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="D44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1409,14 +1237,10 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>07:34</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+          <t>23:19</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -1431,14 +1255,10 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>13:01</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+          <t>07:34</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -1453,14 +1273,10 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>17:16</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>13:01</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -1475,14 +1291,10 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>23:19</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+          <t>17:16</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>